<commit_message>
feat(F-NAR-019): ATOM-AUT.AFF.002-07 Le cacao et le pain de Mila
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.AFF.002-07.xlsx
+++ b/stories/arbres/ATOM-AUT.AFF.002-07.xlsx
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Après le cacao, Mila veut le pain chaud de la boulangerie. Une moufle est coincée dans la manche du manteau vert. Elle la sort, enfile le manteau, sent le pain, raccroche.</t>
+          <t>La vapeur du cacao dessine un nuage sur la vitre. Sur le bord, un éclat de tasse brille, comme une lune. Mila veut le pain de la rue, maintenant. Elle pousse les deux bras d'un coup : la manche avale la moufle. Elle refuse de forcer, pose, enfile le manteau. Merci vécu. Devant la boulangerie, une flaque barre le pas. Elle refuse de foncer. Dans l'eau, l'éclat blanc pointe le pain rond. Ils rentrent. L'éclat de tasse et la lune de farine se regardent.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Deux tasses encore tièdes. Un peu de cacao au fond. La table sent le lait. La veste de papa est sur le dossier. Une moufle sèche sur le radiateur. Mila, tu as fini ton cacao ? Oui, papa. Il était chaud. En ce moment, Mila pose sa tasse. Son manteau vert attend au crochet. On va chercher le pain ? Oui. À la boulangerie. Mila va vers le crochet. Elle prend le manteau vert. Quelque chose est dans la manche. Il y a quelque chose ! Tu peux sortir ce qu'il y a ? Mila tire tout doux. C'est la moufle. Elle est sèche, maintenant. C'est la moufle ! Elle était dans la manche. Maintenant tu peux l'enfiler. Mila passe les manches. Le tissu est doux. Tu veux la moufle ? Oui. Elle est sèche. Papa ouvre la porte. L'air est frais. Ils sortent. À la boulangerie, ça sent le pain chaud. Mila tient la main de papa. J'ai chaud dans le manteau. Oui. Parce que tu l'as pris. La cloche de la porte tinte. Le pain brille derrière la vitre. Tu as vu le pain ? Il est doré. Papa prend le pain. Il le glisse dans un sac. Le sac est un peu chaud. C'est l'heure de rentrer. Oui. On rentre. Ils rentrent. Mila raccroche le manteau au crochet. Le crochet est bas. Mila pose la moufle près du radiateur. Elle est un peu froide, maintenant. Tu as fini de poser la moufle ? Oui, papa. Le manteau est au crochet. Oui. Tu as su.</t>
+          <t>La vapeur du cacao dessine un nuage, sur la vitre. Deux tasses restent tièdes, sur la table. La table sent le lait, et le chocolat. Un cercle brun sèche près de la nappe. La veste de papa pèse sur le dossier. Le radiateur cliquette près du crochet. Papa, mon cacao est fini. Il était bon, le chaud ? Oui, papa. Il reste un peu au fond. Mila pose sa tasse près du cercle brun. Elle lève le bord vers la lumière. Sur le bord, un éclat de tasse brille. C'est un petit éclat blanc, comme une lune. Il brille, papa. C'est un éclat de tasse, Mila. Dehors, l'air sent le pain, par la fente. La fente de la porte laisse passer le chaud. Je veux le pain, maintenant ! Le four de la rue va le sortir. On y va ? On prend le manteau, d'abord. En ce moment, Mila court vers le crochet. Son manteau vert attend, un peu lourd. Elle saisit le manteau vert. Le tissu sent le chaud du radiateur. Je le mets d'un coup ! Elle pousse les deux bras, trop vite. La manche avale la moufle sèche. Le tissu se bloque, contre le pouce. Ça reste coincé ! Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Tu regardes la manche ?</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Deux tasses encore tièdes. Un peu de cacao au fond. La table sent le lait. La veste de papa est sur le dossier. Une moufle sèche sur le radiateur. Mila, tu as fini ton cacao ? Oui, papa. Il était chaud. En ce moment, Mila pose sa tasse. Son manteau vert attend au crochet. On va chercher le pain ? Oui. À la boulangerie. Mila va vers le crochet. Elle prend le manteau vert. Quelque chose est dans la manche. Il y a quelque chose ! Tu peux sortir ce qu'il y a ? Mila tire tout doux. C'est la moufle. Elle est sèche, maintenant. C'est la moufle ! Elle était dans la manche. Maintenant tu peux l'enfiler. Mila passe les manches. Le tissu est doux. Tu veux la moufle ? Oui. Elle est sèche. Papa ouvre la porte. L'air est frais. Ils sortent. À la boulangerie, ça sent le pain chaud. Mila tient la main de papa. J'ai chaud dans le manteau. Oui. Parce que tu l'as pris. La cloche de la porte tinte. Le pain brille derrière la vitre. Tu as vu le pain ? Il est doré. Papa prend le pain. Il le glisse dans un sac. Le sac est un peu chaud. C'est l'heure de rentrer. Oui. On rentre. Ils rentrent. Mila raccroche le manteau au crochet. Le crochet est bas. Mila pose la moufle près du radiateur. Elle est un peu froide, maintenant. Tu as fini de poser la moufle ? Oui, papa. Le manteau est au crochet. Oui. Tu as su.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La vapeur du cacao dessine un nuage, sur la vitre. Deux tasses restent tièdes, sur la table. La table sent le lait, et le chocolat. Un cercle brun sèche près de la nappe. La veste de papa pèse sur le dossier. Le radiateur cliquette près du crochet. Papa, mon cacao est fini. Il était bon, le chaud ? Oui, papa. Il reste un peu au fond. Mila pose sa tasse près du cercle brun. Elle lève le bord vers la lumière. Sur le bord, un &lt;emphasis level="moderate"&gt;éclat de tasse&lt;/emphasis&gt; brille. C'est un petit éclat blanc, comme une lune. Il brille, papa. C'est un éclat de tasse, Mila. Dehors, l'air sent le pain, par la fente. La fente de la porte laisse passer le chaud. Je veux le pain, maintenant ! Le four de la rue va le sortir. On y va ? On prend le manteau, d'abord. En ce moment, Mila court vers le crochet. Son manteau vert attend, un peu lourd. Elle saisit le manteau vert. Le tissu sent le chaud du radiateur. Je le mets d'un coup ! Elle pousse les deux bras, trop vite. La manche avale la moufle sèche. Le tissu se bloque, contre le pouce. Ça reste coincé ! Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Tu regardes la manche ?&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Florian veut aller chercher le pain. Papa ouvre la porte de l'entrée. L'air est frais. Papa dit : avant de sortir, on prend le &lt;emphasis&gt;manteau&lt;/emphasis&gt;. Florian prend son manteau vert. Il passe les manches. Le tissu est doux. Ils sortent. À la boulangerie, ça sent le pain chaud. Florian tient la main de papa. Puis ils rentrent. Papa dit : en rentrant, le manteau va à sa place. Florian raccroche le manteau au crochet. Le crochet est bas. Florian dit : manteau pour sortir. Manteau à sa place en rentrant. Papa sourit. Les chaussures restent près de la porte. Parce qu'il a pris le manteau, Florian a eu chaud dehors. En rentrant, le manteau a sa place. [pause]</t>
+          <t>La vapeur du cacao dessine un nuage, sur la vitre. Deux tasses restent tièdes, sur la table. La table sent le lait, et le chocolat. Un cercle brun sèche près de la nappe. La veste de papa pèse sur le dossier. Le radiateur cliquette près du crochet. Papa, mon cacao est fini. Il était bon, le chaud ? Oui, papa. Il reste un peu au fond. Mila pose sa tasse près du cercle brun. Elle lève le bord vers la lumière. Sur le bord, un &lt;emphasis&gt;éclat de tasse&lt;/emphasis&gt; brille. C'est un petit éclat blanc, comme une lune. Il brille, papa. C'est un éclat de tasse, Mila. Dehors, l'air sent le pain, par la fente. La fente de la porte laisse passer le chaud. Je veux le pain, maintenant ! Le four de la rue va le sortir. On y va ? On prend le manteau, d'abord. En ce moment, Mila court vers le crochet. Son manteau vert attend, un peu lourd. Elle saisit le manteau vert. Le tissu sent le chaud du radiateur. Je le mets d'un coup ! Elle pousse les deux bras, trop vite. La manche avale la moufle sèche. Le tissu se bloque, contre le pouce. Ça reste coincé ! Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Tu regardes la manche ? [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>manteau</t>
+          <t>éclat de tasse</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,71 +1321,52 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_le_pain_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Deux tasses encore tièdes.
-narrateur|Un peu de cacao au fond.
-narrateur|La table sent le lait.
-narrateur|La veste de papa est sur le dossier.
-narrateur|Une moufle sèche sur le radiateur.
-papa|Mila, tu as fini ton cacao ?
+          <t>narrateur|La vapeur du cacao dessine un nuage, sur la vitre.
+narrateur|Deux tasses restent tièdes, sur la table.
+narrateur|La table sent le lait, et le chocolat.
+narrateur|Un cercle brun sèche près de la nappe.
+narrateur|La veste de papa pèse sur le dossier.
+narrateur|Le radiateur cliquette près du crochet.
+enfant-f|Papa, mon cacao est fini.
+papa|Il était bon, le chaud ?
 enfant-f|Oui, papa.
-enfant-f|Il était chaud.
-narrateur|En ce moment, Mila pose sa tasse.
-narrateur|Son manteau vert attend au crochet.
-enfant-f|On va chercher le pain ?
-papa|Oui.
-papa|À la boulangerie.
-narrateur|Mila va vers le crochet.
-narrateur|Elle prend le manteau vert.
-narrateur|Quelque chose est dans la manche.
-enfant-f|Il y a quelque chose !
-papa|Tu peux sortir ce qu'il y a ?
-narrateur|Mila tire tout doux.
-narrateur|C'est la moufle.
-narrateur|Elle est sèche, maintenant.
-enfant-f|C'est la moufle !
-papa|Elle était dans la manche.
-papa|Maintenant tu peux l'enfiler.
-narrateur|Mila passe les manches.
-narrateur|Le tissu est doux.
-papa|Tu veux la moufle ?
-enfant-f|Oui.
-enfant-f|Elle est sèche.
-narrateur|Papa ouvre la porte.
-narrateur|L'air est frais.
-narrateur|Ils sortent.
-narrateur|À la boulangerie, ça sent le pain chaud.
-narrateur|Mila tient la main de papa.
-enfant-f|J'ai chaud dans le manteau.
-papa|Oui.
-papa|Parce que tu l'as pris.
-narrateur|La cloche de la porte tinte.
-narrateur|Le pain brille derrière la vitre.
-papa|Tu as vu le pain ?
-enfant-f|Il est doré.
-narrateur|Papa prend le pain.
-narrateur|Il le glisse dans un sac.
-narrateur|Le sac est un peu chaud.
-papa|C'est l'heure de rentrer.
-enfant-f|Oui.
-enfant-f|On rentre.
-narrateur|Ils rentrent.
-narrateur|Mila raccroche le manteau au crochet.
-narrateur|Le crochet est bas.
-narrateur|Mila pose la moufle près du radiateur.
-narrateur|Elle est un peu froide, maintenant.
-papa|Tu as fini de poser la moufle ?
-enfant-f|Oui, papa.
-enfant-f|Le manteau est au crochet.
-papa|Oui.
-papa|Tu as su.</t>
+enfant-f|Il reste un peu au fond.
+narrateur|Mila pose sa tasse près du cercle brun.
+narrateur|Elle lève le bord vers la lumière.
+narrateur|Sur le bord, un éclat de tasse brille.
+narrateur|C'est un petit éclat blanc, comme une lune.
+enfant-f|Il brille, papa.
+papa|C'est un éclat de tasse, Mila.
+narrateur|Dehors, l'air sent le pain, par la fente.
+narrateur|La fente de la porte laisse passer le chaud.
+enfant-f|Je veux le pain, maintenant !
+papa|Le four de la rue va le sortir.
+enfant-f|On y va ?
+papa|On prend le manteau, d'abord.
+narrateur|En ce moment, Mila court vers le crochet.
+narrateur|Son manteau vert attend, un peu lourd.
+narrateur|Elle saisit le manteau vert.
+narrateur|Le tissu sent le chaud du radiateur.
+enfant-f|Je le mets d'un coup !
+narrateur|Elle pousse les deux bras, trop vite.
+narrateur|La manche avale la moufle sèche.
+narrateur|Le tissu se bloque, contre le pouce.
+enfant-f|Ça reste coincé !
+narrateur|Le sourire de Mila disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+papa|Tu regardes la manche ?</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>tasses,porte</t>
+          <t>tasses,vapeur</t>
         </is>
       </c>
     </row>
@@ -1412,17 +1393,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Avant de sortir, que prend Mila ?</t>
+          <t>Mila tient le manteau. Avant de sortir, que prend Mila ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Avant de sortir, que prend Mila ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Mila tient le &lt;emphasis level="moderate"&gt;manteau&lt;/emphasis&gt;. Avant de sortir, que prend Mila ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Avant de &lt;emphasis&gt;sortir&lt;/emphasis&gt;, que prend Florian ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Mila tient le &lt;emphasis&gt;manteau&lt;/emphasis&gt;. Avant de sortir, que prend Mila ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1485,7 +1466,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1496,7 +1477,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.22</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1511,38 +1492,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AH3" s="2" t="inlineStr">
         <is>
-          <t>sortir</t>
+          <t>manteau</t>
         </is>
       </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1557,22 +1538,23 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=elle_prend_le_manteau; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Avant de sortir, que prend Mila ?</t>
+          <t>narrateur|Mila tient le manteau.
+narrateur|Avant de sortir, que prend Mila ?</t>
         </is>
       </c>
     </row>
@@ -1599,17 +1581,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Mila a pris le manteau vert. Elle l'a mis pour chercher le pain. Dehors, elle a eu chaud. En rentrant, elle l'a raccroché. Tu as pris le manteau pour sortir. Il est à sa place. Oui. Près de la moufle.</t>
+          <t>Papa s'accroupit à la même hauteur. Mila refuse de tirer plus fort. Je sors la moufle. Elle tire le tissu coincé, sans forcer. La moufle glisse, un peu froide. Elle était dans la manche. Tu la poses où ? Près du radiateur. Mila pose la moufle sèche. Le radiateur cliquette sous la laine. Et le manteau ? Je le mets. Elle passe une manche, puis l'autre. Le tissu vert gratte un peu, aux poignets. J'ai les bras dedans. Tu as fini tes manches ? Oui, papa. Mila boutonne le bas, un par un. C'est fermé. Merci, Mila. Papa ouvre la porte de l'entrée. L'air frais pique les joues. On va au pain ? Oui, à la boulangerie.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Mila a pris le manteau vert. Elle l'a mis pour chercher le pain. Dehors, elle a eu chaud. En rentrant, elle l'a raccroché. Tu as pris le manteau pour sortir. Il est à sa place. Oui. Près de la moufle.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Papa s'accroupit à la même hauteur. Mila refuse de tirer plus fort. Je sors la moufle. Elle tire le tissu coincé, sans forcer. La moufle glisse, un peu froide. Elle était dans la manche. Tu la poses où ? Près du radiateur. Mila pose la moufle sèche. Le radiateur cliquette sous la laine. Et le &lt;emphasis level="moderate"&gt;manteau&lt;/emphasis&gt; ? Je le mets. Elle passe une manche, puis l'autre. Le tissu vert gratte un peu, aux poignets. J'ai les bras dedans. Tu as fini tes manches ? Oui, papa. Mila boutonne le bas, un par un. C'est fermé. Merci, Mila. Papa ouvre la porte de l'entrée. L'air frais pique les joues. On va au pain ? Oui, à la boulangerie.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Florian a pris le &lt;emphasis&gt;manteau&lt;/emphasis&gt; pour sortir. En rentrant, il l'a raccroché. [pause]</t>
+          <t>Papa s'accroupit à la même hauteur. Mila refuse de tirer plus fort. Je sors la moufle. Elle tire le tissu coincé, sans forcer. La moufle glisse, un peu froide. Elle était dans la manche. Tu la poses où ? Près du radiateur. Mila pose la moufle sèche. Le radiateur cliquette sous la laine. Et le &lt;emphasis&gt;manteau&lt;/emphasis&gt; ? Je le mets. Elle passe une manche, puis l'autre. Le tissu vert gratte un peu, aux poignets. J'ai les bras dedans. Tu as fini tes manches ? Oui, papa. Mila boutonne le bas, un par un. C'est fermé. Merci, Mila. Papa ouvre la porte de l'entrée. L'air frais pique les joues. On va au pain ? Oui, à la boulangerie. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1667,7 +1649,7 @@
         <v>0.92</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.2</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1704,16 +1686,16 @@
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1738,19 +1720,40 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=confirmation; intention=faire_vivre_le_geste; emotion=concentration puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=une_manche_puis_l_autre; tempo=naturel; sourire=léger; respiration=fluide</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Mila a pris le manteau vert.
-narrateur|Elle l'a mis pour chercher le pain.
-narrateur|Dehors, elle a eu chaud.
-narrateur|En rentrant, elle l'a raccroché.
-papa|Tu as pris le manteau pour sortir.
-enfant-f|Il est à sa place.
-papa|Oui.
-papa|Près de la moufle.</t>
+          <t>narrateur|Papa s'accroupit à la même hauteur.
+narrateur|Mila refuse de tirer plus fort.
+enfant-f|Je sors la moufle.
+narrateur|Elle tire le tissu coincé, sans forcer.
+narrateur|La moufle glisse, un peu froide.
+enfant-f|Elle était dans la manche.
+papa|Tu la poses où ?
+enfant-f|Près du radiateur.
+narrateur|Mila pose la moufle sèche.
+narrateur|Le radiateur cliquette sous la laine.
+papa|Et le manteau ?
+enfant-f|Je le mets.
+narrateur|Elle passe une manche, puis l'autre.
+narrateur|Le tissu vert gratte un peu, aux poignets.
+enfant-f|J'ai les bras dedans.
+papa|Tu as fini tes manches ?
+enfant-f|Oui, papa.
+narrateur|Mila boutonne le bas, un par un.
+enfant-f|C'est fermé.
+papa|Merci, Mila.
+narrateur|Papa ouvre la porte de l'entrée.
+narrateur|L'air frais pique les joues.
+enfant-f|On va au pain ?
+papa|Oui, à la boulangerie.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>tissu,radiateur</t>
         </is>
       </c>
     </row>
@@ -1777,17 +1780,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Mila pose le pain sur la table. Le sac est encore un peu chaud. Papa ferme la porte. Tu as fini de poser le pain ? Oui, papa. Les tasses sont froides, maintenant. Le manteau vert reste au crochet. On goûtera le pain tout à l'heure. Il sent bon. Oui. Il sent le chaud. Mila pose une main sur le pain. Le sac craque un peu.</t>
+          <t>Ils marchent sur les dalles froides. Le manteau tape contre les genoux de Mila. Une odeur de four glisse dans la rue. Tu tiens ma main ? Oui, papa. J'ai chaud dans le manteau. Oui, le vent est froid. Je le vois ! Derrière la vitre, un pain rond attend. Je cours le prendre ! Mila veut foncer vers la porte. Une flaque barre le pas, devant le seuil. Le sourire de Mila se serre. Ça serre, dans son ventre. Je n'aime pas ça. Mila refuse de foncer. Attends, je regarde. Personne ne donne la réponse. Mila observe le pain, écoute la rue. Dans la flaque, un éclat blanc tremble. Comme l'éclat de tasse, papa ! Tu le vois, celui-là ? Oui, papa. Il pointe le pain rond. Elle contourne la flaque, lentement. La cloche de la porte tinte. Ça sent le chaud, et la farine. Tu tiens le sac ? Oui, il est un peu chaud.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Mila pose le pain sur la table. Le sac est encore un peu chaud. Papa ferme la porte. Tu as fini de poser le pain ? Oui, papa. Les tasses sont froides, maintenant. Le manteau vert reste au crochet. On goûtera le pain tout à l'heure. Il sent bon. Oui. Il sent le chaud. Mila pose une main sur le pain. Le sac craque un peu.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Ils marchent sur les dalles froides. Le manteau tape contre les genoux de Mila. Une odeur de four glisse dans la rue. Tu tiens ma main ? Oui, papa. J'ai chaud dans le manteau. Oui, le vent est froid. Je le vois ! Derrière la vitre, un pain rond attend. Je cours le prendre ! Mila veut foncer vers la porte. Une flaque barre le pas, devant le seuil. Le sourire de Mila se serre. Ça serre, dans son ventre. Je n'aime pas ça. Mila refuse de foncer. Attends, je regarde. Personne ne donne la réponse. Mila observe le pain, écoute la rue. Dans la flaque, un éclat blanc tremble. Comme l'&lt;emphasis level="moderate"&gt;éclat de tasse&lt;/emphasis&gt;, papa ! Tu le vois, celui-là ? Oui, papa. Il pointe le pain rond. Elle contourne la flaque, lentement. La cloche de la porte tinte. Ça sent le chaud, et la farine. Tu tiens le sac ? Oui, il est un peu chaud.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Florian pose &lt;emphasis&gt;le&lt;/emphasis&gt; pain sur la table. Papa ferme la porte. [pause]</t>
+          <t>Ils marchent sur les dalles froides. Le manteau tape contre les genoux de Mila. Une odeur de four glisse dans la rue. Tu tiens ma main ? Oui, papa. J'ai chaud dans le manteau. Oui, le vent est froid. Je le vois ! Derrière la vitre, un pain rond attend. Je cours le prendre ! Mila veut foncer vers la porte. Une flaque barre le pas, devant le seuil. Le sourire de Mila se serre. Ça serre, dans son ventre. Je n'aime pas ça. Mila refuse de foncer. Attends, je regarde. Personne ne donne la réponse. Mila observe le pain, écoute la rue. Dans la flaque, un éclat blanc tremble. Comme l'&lt;emphasis&gt;éclat de tasse&lt;/emphasis&gt;, papa ! Tu le vois, celui-là ? Oui, papa. Il pointe le pain rond. Elle contourne la flaque, lentement. La cloche de la porte tinte. Ça sent le chaud, et la farine. Tu tiens le sac ? Oui, il est un peu chaud. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1834,7 +1837,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1842,10 +1845,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1868,30 +1871,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>le</t>
+          <t>éclat de tasse</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1900,10 +1903,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1914,22 +1917,47 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_dans_la_flaque; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Mila pose le pain sur la table.
-narrateur|Le sac est encore un peu chaud.
-narrateur|Papa ferme la porte.
-papa|Tu as fini de poser le pain ?
+          <t>narrateur|Ils marchent sur les dalles froides.
+narrateur|Le manteau tape contre les genoux de Mila.
+narrateur|Une odeur de four glisse dans la rue.
+papa|Tu tiens ma main ?
 enfant-f|Oui, papa.
-narrateur|Les tasses sont froides, maintenant.
-narrateur|Le manteau vert reste au crochet.
-papa|On goûtera le pain tout à l'heure.
-enfant-f|Il sent bon.
-papa|Oui.
-papa|Il sent le chaud.
-narrateur|Mila pose une main sur le pain.
-narrateur|Le sac craque un peu.</t>
+enfant-f|J'ai chaud dans le manteau.
+papa|Oui, le vent est froid.
+enfant-f|Je le vois !
+narrateur|Derrière la vitre, un pain rond attend.
+enfant-f|Je cours le prendre !
+narrateur|Mila veut foncer vers la porte.
+narrateur|Une flaque barre le pas, devant le seuil.
+narrateur|Le sourire de Mila se serre.
+narrateur|Ça serre, dans son ventre.
+enfant-f|Je n'aime pas ça.
+narrateur|Mila refuse de foncer.
+enfant-f|Attends, je regarde.
+narrateur|Personne ne donne la réponse.
+narrateur|Mila observe le pain, écoute la rue.
+narrateur|Dans la flaque, un éclat blanc tremble.
+enfant-f|Comme l'éclat de tasse, papa !
+papa|Tu le vois, celui-là ?
+enfant-f|Oui, papa.
+enfant-f|Il pointe le pain rond.
+narrateur|Elle contourne la flaque, lentement.
+narrateur|La cloche de la porte tinte.
+narrateur|Ça sent le chaud, et la farine.
+papa|Tu tiens le sac ?
+enfant-f|Oui, il est un peu chaud.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>dalles,cloche</t>
         </is>
       </c>
     </row>
@@ -1956,17 +1984,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai pris le manteau pour le pain. En rentrant, je l'ai raccroché. Bravo, Mila. Le cacao a laissé une petite odeur.</t>
+          <t>Ils rentrent dans la cuisine tiède. Mila raccroche le manteau vert, au crochet. Le crochet est bas, sous la veste de papa. Papa ferme la porte de l'entrée. Le pain est là. Oui, près des tasses. Mila pose le sac chaud sur la table. Le cercle brun touche le papier. Mon éclat de tasse, papa. Sur le bord, l'éclat de tasse brille. Sur la croûte, la lune de farine brille aussi. Ils se regardent. Tu les sens, le cacao et le pain ? Oui, papa. Le pain sent le chaud. L'éclat de tasse reste sur le bord.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai pris le manteau pour le pain. En rentrant, je l'ai raccroché. Bravo, Mila. Le cacao a laissé une petite odeur.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils rentrent dans la cuisine tiède. Mila raccroche le manteau vert, au crochet. Le crochet est bas, sous la veste de papa. Papa ferme la porte de l'entrée. Le pain est là. Oui, près des tasses. Mila pose le sac chaud sur la table. Le cercle brun touche le papier. Mon &lt;emphasis level="moderate"&gt;éclat de tasse&lt;/emphasis&gt;, papa. Sur le bord, l'éclat de tasse brille. Sur la croûte, la lune de farine brille aussi. Ils se regardent. Tu les sens, le cacao et le pain ? Oui, papa. Le pain sent le chaud. L'éclat de tasse reste sur le bord.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils rentrent dans la cuisine tiède. Mila raccroche le manteau vert, au crochet. Le crochet est bas, sous la veste de papa. Papa ferme la porte de l'entrée. Le pain est là. Oui, près des tasses. Mila pose le sac chaud sur la table. Le cercle brun touche le papier. Mon &lt;emphasis&gt;éclat de tasse&lt;/emphasis&gt;, papa. Sur le bord, l'éclat de tasse brille. Sur la croûte, la lune de farine brille aussi. Ils se regardent. Tu les sens, le cacao et le pain ? Oui, papa. Le pain sent le chaud. L'éclat de tasse reste sur le bord.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2013,7 +2041,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2021,7 +2049,7 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
         <v>1.28</v>
@@ -2033,12 +2061,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2047,17 +2075,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de tasse</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2066,11 +2098,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2079,27 +2111,48 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_de_la_tasse_est_sur_le_pain; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|J'ai pris le manteau pour le pain.
-enfant-f|En rentrant, je l'ai raccroché.
-papa|Bravo, Mila.
-narrateur|Le cacao a laissé une petite odeur.</t>
+          <t>narrateur|Ils rentrent dans la cuisine tiède.
+narrateur|Mila raccroche le manteau vert, au crochet.
+narrateur|Le crochet est bas, sous la veste de papa.
+narrateur|Papa ferme la porte de l'entrée.
+enfant-f|Le pain est là.
+papa|Oui, près des tasses.
+narrateur|Mila pose le sac chaud sur la table.
+narrateur|Le cercle brun touche le papier.
+enfant-f|Mon éclat de tasse, papa.
+narrateur|Sur le bord, l'éclat de tasse brille.
+narrateur|Sur la croûte, la lune de farine brille aussi.
+enfant-f|Ils se regardent.
+papa|Tu les sens, le cacao et le pain ?
+enfant-f|Oui, papa.
+enfant-f|Le pain sent le chaud.
+narrateur|L'éclat de tasse reste sur le bord.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>pain,tasse</t>
         </is>
       </c>
     </row>
@@ -2120,7 +2173,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2212,6 +2265,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>